<commit_message>
Fix: deduplicate prolongations by id+month (keep first AM)
</commit_message>
<xml_diff>
--- a/prolongation_report.xlsx
+++ b/prolongation_report.xlsx
@@ -717,7 +717,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>3 377 742</t>
+          <t>2 982 484</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>50.4%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -754,22 +754,22 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>3 647 436</t>
+          <t>3 414 632</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2 194 461</t>
+          <t>1 981 262</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>60.2%</t>
+          <t>58.0%</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>1 796 704</t>
+          <t>1 401 446</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -939,17 +939,17 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>3 820 836</t>
+          <t>3 686 851</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>3 162 695</t>
+          <t>3 014 655</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>81.8%</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1132,22 +1132,22 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>11 761 148</t>
+          <t>11 133 085</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>6 119 964</t>
+          <t>5 906 765</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>52.0%</t>
+          <t>53.1%</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>5 818 845</t>
+          <t>5 423 588</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>8.3%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
@@ -1317,17 +1317,17 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>3 680 853</t>
+          <t>3 546 868</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>1 885 686</t>
+          <t>1 737 646</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>51.2%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1637,12 +1637,12 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>35.1%</t>
+          <t>46.6%</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>49.7%</t>
+          <t>44.9%</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>79.4%</t>
+          <t>73.0%</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fix: coef=nan instead of 0 when no base (analytically correct)
</commit_message>
<xml_diff>
--- a/prolongation_report.xlsx
+++ b/prolongation_report.xlsx
@@ -1510,22 +1510,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1734,17 +1734,17 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1776,27 +1776,27 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
@@ -1890,57 +1890,57 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -2150,251 +2150,251 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Федорова Марина Васильевна</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>без А/М</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="11"/>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Коэффициент 2</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
       </c>
-      <c r="G15" s="1" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
       </c>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
       </c>
-      <c r="I15" s="1" t="inlineStr">
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
       </c>
-      <c r="J15" s="1" t="inlineStr">
+      <c r="J13" s="1" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
       </c>
-      <c r="K15" s="1" t="inlineStr">
+      <c r="K13" s="1" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
       </c>
-      <c r="L15" s="1" t="inlineStr">
+      <c r="L13" s="1" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
       </c>
-      <c r="M15" s="1" t="inlineStr">
+      <c r="M13" s="1" t="inlineStr">
         <is>
           <t>2023-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Васильев Артем Александрович</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>18.7%</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>70.8%</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>11.0%</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>5.7%</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>7.2%</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>48.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Иванова Мария Сергеевна</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Васильев Артем Александрович</t>
+          <t>Кузнецов Михаил Иванович</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>18.7%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>70.8%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -2404,44 +2404,44 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>5.7%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>7.2%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>48.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Иванова Мария Сергеевна</t>
+          <t>Михайлов Андрей Сергеевич</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -2456,22 +2456,22 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -2481,12 +2481,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
@@ -2501,14 +2501,14 @@
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Кузнецов Михаил Иванович</t>
+          <t>Попова Екатерина Николаевна</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>50.6%</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -2558,29 +2558,29 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>62.2%</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>19.0%</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Михайлов Андрей Сергеевич</t>
+          <t>Смирнова Ольга Владимировна</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -2590,32 +2590,32 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>115.1%</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>Нет данных</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>51.6%</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>155.3%</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
@@ -2635,24 +2635,24 @@
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>39.8%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Петрова Анна Дмитриевна</t>
+          <t>Соколова Анастасия Викторовна</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>67.9%</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>21.6%</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2701,341 +2701,6 @@
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Попова Екатерина Николаевна</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>19.1%</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>50.6%</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>62.2%</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Смирнова Ольга Владимировна</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>115.1%</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>51.6%</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>155.3%</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L22" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M22" s="6" t="inlineStr">
-        <is>
-          <t>39.8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Соколова Анастасия Викторовна</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>67.9%</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>21.6%</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M23" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Федорова Марина Васильевна</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M24" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>без А/М</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L25" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M25" s="6" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
@@ -3043,8 +2708,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:M14"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A12:M12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add summary sheet 'Итоги' with dept by month + managers by year
</commit_message>
<xml_diff>
--- a/prolongation_report.xlsx
+++ b/prolongation_report.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Весь отдел" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Менеджеры за год" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Менеджеры по месяцам" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Итоги" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Весь отдел" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Менеджеры за год" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Менеджеры по месяцам" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +32,13 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00999999"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B942"/>
       </patternFill>
     </fill>
   </fills>
@@ -153,20 +164,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -532,6 +547,996 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Весь отдел — по месяцам</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="n"/>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Месяц</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации в первый месяц</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации через месяц</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>к пролонгации</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>пролонгировано</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Коэффициент</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>к пролонгации</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>пролонгировано</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Коэффициент</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>5 986 767</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>2 677 022</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>44.7%</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>545 022</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>73 380</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>13.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>2 549 076</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>1 880 945</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>73.8%</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2 890 043</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>262 620</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>9.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>1 899 333</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>1 271 739</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>67.0%</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>760 840</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>122 999</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>16.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2 982 484</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>1 501 923</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>50.4%</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>627 735</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>57 940</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>9.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>3 414 632</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>1 981 262</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>58.0%</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>1 401 446</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>1 274 626</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>333 068</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>26.1%</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>1 015 068</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>38 632</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>2 625 983</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>1 390 411</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>52.9%</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>1 020 326</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>108 285</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>10.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>1 936 916</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>943 679</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>48.7%</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>1 452 500</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>52 315</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>3.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>3 241 978</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>1 086 504</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>33.5%</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>755 740</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>3 686 851</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>3 014 655</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>81.8%</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>2 183 145</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>245 379</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>1 567 140</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>811 594</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>51.8%</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>1 130 393</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>21 400</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>2 434 795</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>1 325 978</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>54.5%</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>735 958</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>114 440</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Менеджеры — итог за 2023 год</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации в первый месяц</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации через месяц</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>к пролонгации</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>пролонгировано</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Коэффициент</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>к пролонгации</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>пролонгировано</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Коэффициент</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Васильев Артем Александрович</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>11 133 085</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>5 906 765</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>53.1%</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>5 423 588</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>482 442</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Иванова Мария Сергеевна</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>4 727 657</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>1 660 096</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>35.1%</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>2 503 865</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Кузнецов Михаил Иванович</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>982 724</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>470 183</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>47.8%</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>167 675</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Михайлов Андрей Сергеевич</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>3 361 834</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>2 235 422</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>66.5%</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>1 056 005</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Петрова Анна Дмитриевна</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>98 492</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>109 443</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>111.1%</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Попова Екатерина Николаевна</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>3 546 868</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>1 737 646</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>49.0%</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>1 750 920</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>241 399</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>13.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Смирнова Ольга Владимировна</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>2 951 205</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>2 124 958</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>72.0%</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>803 501</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>203 825</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>25.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Соколова Анастасия Викторовна</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>6 798 715</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>3 974 268</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>58.5%</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>2 812 662</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>169 725</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>6.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Федорова Марина Васильевна</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>без А/М</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>← Вставьте график здесь</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -545,498 +1550,498 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Месяц</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Пролонгации в первый месяц</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="4" t="n"/>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Пролонгации через месяц</t>
         </is>
       </c>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="4" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>5 986 767</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>2 677 022</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>44.7%</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>545 022</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>73 380</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>13.5%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>2 549 076</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>1 880 945</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>73.8%</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>2 890 043</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>262 620</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>9.1%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>1 899 333</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>1 271 739</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>67.0%</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>760 840</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>122 999</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>16.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>2 982 484</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>1 501 923</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>50.4%</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>627 735</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>57 940</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>9.2%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>3 414 632</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>1 981 262</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>58.0%</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>1 401 446</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>1 274 626</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>333 068</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>26.1%</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>1 015 068</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>38 632</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>3.8%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>2 625 983</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>1 390 411</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>52.9%</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>1 020 326</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>108 285</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>10.6%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>1 936 916</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>943 679</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>48.7%</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>1 452 500</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>52 315</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>3.6%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>3 241 978</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>1 086 504</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>33.5%</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>755 740</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>3 686 851</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>3 014 655</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>81.8%</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>2 183 145</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>245 379</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>11.2%</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>1 567 140</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>811 594</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>51.8%</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>1 130 393</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>21 400</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>1.9%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>2023-12</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>2 434 795</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>1 325 978</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>54.5%</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>735 958</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>114 440</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>15.5%</t>
         </is>
@@ -1052,7 +2057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1071,424 +2076,424 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Пролонгации в первый месяц</t>
         </is>
       </c>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="4" t="n"/>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Пролонгации через месяц</t>
         </is>
       </c>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="4" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="5" t="n"/>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Васильев Артем Александрович</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>11 133 085</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>5 906 765</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>53.1%</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>5 423 588</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>482 442</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Иванова Мария Сергеевна</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>4 727 657</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>1 660 096</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>35.1%</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>2 503 865</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Кузнецов Михаил Иванович</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>982 724</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>470 183</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>47.8%</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>167 675</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Михайлов Андрей Сергеевич</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>3 361 834</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>2 235 422</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>66.5%</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>1 056 005</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Петрова Анна Дмитриевна</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>98 492</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>109 443</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>111.1%</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Попова Екатерина Николаевна</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>3 546 868</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>1 737 646</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>49.0%</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>1 750 920</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>241 399</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>13.8%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Смирнова Ольга Владимировна</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>2 951 205</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>2 124 958</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>72.0%</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>803 501</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>203 825</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>25.4%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Соколова Анастасия Викторовна</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>6 798 715</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>3 974 268</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>58.5%</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>2 812 662</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>169 725</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>6.0%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Федорова Марина Васильевна</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>без А/М</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
@@ -1504,7 +2509,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1529,622 +2534,622 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Коэффициент 1</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
-      <c r="I1" s="3" t="n"/>
-      <c r="J1" s="3" t="n"/>
-      <c r="K1" s="3" t="n"/>
-      <c r="L1" s="3" t="n"/>
-      <c r="M1" s="4" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="3" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
       </c>
-      <c r="L2" s="1" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
       </c>
-      <c r="M2" s="1" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>2023-12</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Васильев Артем Александрович</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>55.6%</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>115.6%</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>62.7%</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>46.6%</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>44.9%</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>38.9%</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>58.5%</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>47.8%</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>17.2%</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>88.7%</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
+      <c r="L3" s="7" t="inlineStr">
         <is>
           <t>62.1%</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>32.4%</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Иванова Мария Сергеевна</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>27.0%</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>44.6%</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>27.8%</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>47.3%</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>54.1%</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>99.9%</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Кузнецов Михаил Иванович</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>126.6%</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>84.7%</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
         <is>
           <t>130.9%</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>47.4%</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="M5" s="7" t="inlineStr">
         <is>
           <t>27.4%</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Михайлов Андрей Сергеевич</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>68.8%</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>90.4%</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>243.1%</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>109.9%</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>119.0%</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>119.8%</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>44.9%</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Петрова Анна Дмитриевна</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
         <is>
           <t>111.1%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Попова Екатерина Николаевна</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>44.1%</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>68.5%</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>28.9%</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>75.7%</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>9.6%</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>48.0%</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J8" s="7" t="inlineStr">
         <is>
           <t>45.4%</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>73.0%</t>
         </is>
       </c>
-      <c r="L8" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
         <is>
           <t>60.0%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Смирнова Ольга Владимировна</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>74.3%</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>96.6%</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>38.2%</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
         <is>
           <t>37.3%</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="7" t="inlineStr">
         <is>
           <t>76.5%</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>104.7%</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>83.6%</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="M9" s="7" t="inlineStr">
         <is>
           <t>36.1%</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Соколова Анастасия Викторовна</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>42.7%</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>23.5%</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>93.9%</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>106.6%</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>23.7%</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>76.6%</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>61.9%</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>54.1%</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>29.5%</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>84.2%</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>17.9%</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>79.1%</t>
         </is>
@@ -2152,555 +3157,555 @@
     </row>
     <row r="11"/>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Коэффициент 2</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="4" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="3" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Менеджер</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>2023-01</t>
         </is>
       </c>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>2023-02</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>2023-03</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>2023-04</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>2023-05</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>2023-06</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>2023-07</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>2023-08</t>
         </is>
       </c>
-      <c r="J13" s="1" t="inlineStr">
+      <c r="J13" s="4" t="inlineStr">
         <is>
           <t>2023-09</t>
         </is>
       </c>
-      <c r="K13" s="1" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>2023-10</t>
         </is>
       </c>
-      <c r="L13" s="1" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>2023-11</t>
         </is>
       </c>
-      <c r="M13" s="1" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>2023-12</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Васильев Артем Александрович</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>18.7%</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>70.8%</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>11.0%</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>5.7%</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>7.2%</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
         <is>
           <t>48.5%</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Иванова Мария Сергеевна</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Кузнецов Михаил Иванович</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="L16" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Михайлов Андрей Сергеевич</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L17" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Попова Екатерина Николаевна</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>19.1%</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>50.6%</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>62.2%</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="L18" s="7" t="inlineStr">
         <is>
           <t>19.0%</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
+      <c r="M18" s="7" t="inlineStr">
         <is>
           <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Смирнова Ольга Владимировна</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>115.1%</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>51.6%</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>155.3%</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L19" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
         <is>
           <t>39.8%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Соколова Анастасия Викторовна</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>67.9%</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>21.6%</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>

</xml_diff>

<commit_message>
Add dept yearly total row to Итоги sheet
</commit_message>
<xml_diff>
--- a/prolongation_report.xlsx
+++ b/prolongation_report.xlsx
@@ -164,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,6 +179,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -547,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1070,172 +1073,172 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Итого за 2023 год</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>33 600 579</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>18 218 781</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>54.2%</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>14 518 215</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>1 097 391</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>7.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Менеджеры — итог за 2023 год</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="3" t="n"/>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Менеджер</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Пролонгации в первый месяц</t>
-        </is>
-      </c>
+      <c r="B18" s="2" t="n"/>
       <c r="C18" s="2" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Пролонгации через месяц</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="3" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Менеджер</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации в первый месяц</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Пролонгации через месяц</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>к пролонгации</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>пролонгировано</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>Коэффициент</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Васильев Артем Александрович</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>11 133 085</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>5 906 765</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>53.1%</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>5 423 588</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>482 442</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Иванова Мария Сергеевна</t>
+          <t>Васильев Артем Александрович</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>4 727 657</t>
+          <t>11 133 085</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>1 660 096</t>
+          <t>5 906 765</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>35.1%</t>
+          <t>53.1%</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>2 503 865</t>
+          <t>5 423 588</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>482 442</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.9%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Кузнецов Михаил Иванович</t>
+          <t>Иванова Мария Сергеевна</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>982 724</t>
+          <t>4 727 657</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>470 183</t>
+          <t>1 660 096</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>47.8%</t>
+          <t>35.1%</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>167 675</t>
+          <t>2 503 865</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -1252,27 +1255,27 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Михайлов Андрей Сергеевич</t>
+          <t>Кузнецов Михаил Иванович</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>3 361 834</t>
+          <t>982 724</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>2 235 422</t>
+          <t>470 183</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>66.5%</t>
+          <t>47.8%</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>1 056 005</t>
+          <t>167 675</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -1289,228 +1292,265 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Петрова Анна Дмитриевна</t>
+          <t>Михайлов Андрей Сергеевич</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>98 492</t>
+          <t>3 361 834</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>109 443</t>
+          <t>2 235 422</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>111.1%</t>
+          <t>66.5%</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
+          <t>1 056 005</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>0.0%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Попова Екатерина Николаевна</t>
+          <t>Петрова Анна Дмитриевна</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>3 546 868</t>
+          <t>98 492</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>1 737 646</t>
+          <t>109 443</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>49.0%</t>
+          <t>111.1%</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>1 750 920</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>241 399</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>13.8%</t>
+          <t>Нет данных</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Смирнова Ольга Владимировна</t>
+          <t>Попова Екатерина Николаевна</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>2 951 205</t>
+          <t>3 546 868</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>2 124 958</t>
+          <t>1 737 646</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>72.0%</t>
+          <t>49.0%</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>803 501</t>
+          <t>1 750 920</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>203 825</t>
+          <t>241 399</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>25.4%</t>
+          <t>13.8%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Соколова Анастасия Викторовна</t>
+          <t>Смирнова Ольга Владимировна</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>6 798 715</t>
+          <t>2 951 205</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>3 974 268</t>
+          <t>2 124 958</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>58.5%</t>
+          <t>72.0%</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>2 812 662</t>
+          <t>803 501</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>169 725</t>
+          <t>203 825</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>6.0%</t>
+          <t>25.4%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Федорова Марина Васильевна</t>
+          <t>Соколова Анастасия Викторовна</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6 798 715</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3 974 268</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>58.5%</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2 812 662</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>169 725</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>6.0%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
+          <t>Федорова Марина Васильевна</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
           <t>без А/М</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Нет данных</t>
-        </is>
-      </c>
-    </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>← Вставьте график здесь</t>
         </is>
@@ -1519,12 +1559,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B19:D19"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E19:G19"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A19:A20"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>